<commit_message>
feat: add Error type column to the observed-data template
The example workbook gets an `Error type` column next to `Error`, filled with
`ASD`. The standard importer configuration does not read it yet, so loading is
unchanged. The test fixture copy stays identical to the template.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/projects/Example/Data/Aciclovir_TimeValuesData.xlsx
+++ b/inst/extdata/projects/Example/Data/Aciclovir_TimeValuesData.xlsx
@@ -536,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B72BA2D-3E1C-441B-963F-68E8C45EAA2D}">
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:V2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
@@ -553,15 +553,16 @@
     <col min="12" max="12" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="20.28515625" customWidth="1"/>
     <col min="14" max="14" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.7109375" customWidth="1"/>
-    <col min="16" max="16" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="34.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" customWidth="1"/>
+    <col min="17" max="17" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -604,29 +605,34 @@
       <c r="N1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Error type</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -669,22 +675,27 @@
       <c r="N2">
         <v>0.3</v>
       </c>
-      <c r="O2">
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>ASD</t>
+        </is>
+      </c>
+      <c r="P2">
         <v>0.01</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>30</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>33</v>
       </c>
-      <c r="S2">
+      <c r="T2">
         <v>153</v>
       </c>
-      <c r="T2">
+      <c r="U2">
         <v>82.5</v>
       </c>
-      <c r="U2">
+      <c r="V2">
         <v>36</v>
       </c>
     </row>
@@ -696,7 +707,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19C774B0-33BA-4040-B2FA-ABDE6C1AB01C}">
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
@@ -713,15 +724,16 @@
     <col min="12" max="12" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="20.28515625" customWidth="1"/>
     <col min="14" max="14" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.7109375" customWidth="1"/>
-    <col min="16" max="16" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="34.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" customWidth="1"/>
+    <col min="17" max="17" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -764,29 +776,34 @@
       <c r="N1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Error type</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -827,11 +844,16 @@
         <v>38</v>
       </c>
       <c r="N2" s="4"/>
-      <c r="P2" t="s">
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>ASD</t>
+        </is>
+      </c>
+      <c r="Q2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>34</v>
       </c>
@@ -874,11 +896,16 @@
       <c r="N3" s="4">
         <v>1.2268330000000001</v>
       </c>
-      <c r="P3" t="s">
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>ASD</t>
+        </is>
+      </c>
+      <c r="Q3" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -921,11 +948,16 @@
       <c r="N4" s="4">
         <v>1.2813950000000001</v>
       </c>
-      <c r="P4" t="s">
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>ASD</t>
+        </is>
+      </c>
+      <c r="Q4" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -968,11 +1000,16 @@
       <c r="N5" s="4">
         <v>1.8176890000000001</v>
       </c>
-      <c r="P5" t="s">
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>ASD</t>
+        </is>
+      </c>
+      <c r="Q5" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -1013,11 +1050,16 @@
         <v>38</v>
       </c>
       <c r="N6" s="4"/>
-      <c r="P6" t="s">
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>ASD</t>
+        </is>
+      </c>
+      <c r="Q6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -1058,11 +1100,16 @@
         <v>38</v>
       </c>
       <c r="N7" s="4"/>
-      <c r="P7" t="s">
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>ASD</t>
+        </is>
+      </c>
+      <c r="Q7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>34</v>
       </c>
@@ -1103,11 +1150,16 @@
         <v>38</v>
       </c>
       <c r="N8" s="4"/>
-      <c r="P8" t="s">
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>ASD</t>
+        </is>
+      </c>
+      <c r="Q8" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -1148,11 +1200,16 @@
         <v>38</v>
       </c>
       <c r="N9" s="4"/>
-      <c r="P9" t="s">
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>ASD</t>
+        </is>
+      </c>
+      <c r="Q9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -1193,11 +1250,16 @@
         <v>38</v>
       </c>
       <c r="N10" s="4"/>
-      <c r="P10" t="s">
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>ASD</t>
+        </is>
+      </c>
+      <c r="Q10" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>34</v>
       </c>
@@ -1238,11 +1300,16 @@
         <v>38</v>
       </c>
       <c r="N11" s="4"/>
-      <c r="P11" t="s">
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>ASD</t>
+        </is>
+      </c>
+      <c r="Q11" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -1283,7 +1350,12 @@
         <v>38</v>
       </c>
       <c r="N12" s="4"/>
-      <c r="P12" t="s">
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>ASD</t>
+        </is>
+      </c>
+      <c r="Q12" t="s">
         <v>39</v>
       </c>
     </row>

</xml_diff>